<commit_message>
normalization: Stackable block tokens; QA: Escambia elections is a gap; tests: URL-uniqueness invariants
</commit_message>
<xml_diff>
--- a/manifest/fl-county-election-pages.xlsx
+++ b/manifest/fl-county-election-pages.xlsx
@@ -4697,58 +4697,46 @@
       <c r="L77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" s="6" t="inlineStr">
         <is>
           <t>Escambia</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
         <is>
           <t>elections</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>https://escambiavotes.gov/</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>found via link "Elections" score=19</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr"/>
-      <c r="J78" s="5" t="inlineStr">
-        <is>
-          <t>confident</t>
-        </is>
-      </c>
-      <c r="K78" s="4" t="inlineStr">
-        <is>
-          <t>[plain] county name 'Escambia' in page; seat 'Pensacola' in page | elections keywords: election | title="EscambiaVotes.gov"</t>
-        </is>
-      </c>
-      <c r="L78" s="2" t="inlineStr"/>
+      <c r="D78" s="6" t="inlineStr"/>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>GAP: folded into SOE homepage — escambiavotes.gov's 'Elections' nav link points back at the homepage, and /elections/ serves the results page; capturing the homepage URL twice would double-count one page</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="H78" s="6" t="inlineStr"/>
+      <c r="I78" s="6" t="inlineStr"/>
+      <c r="J78" s="8" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="K78" s="7" t="inlineStr"/>
+      <c r="L78" s="6" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -18613,249 +18601,248 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D292" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D293" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D294" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D295" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D296" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D297" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D298" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D302" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D303" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D304" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D305" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D306" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D307" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D308" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D309" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D310" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D311" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D312" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D313" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D314" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D315" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D316" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D317" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D318" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D320" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D321" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D322" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D323" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D324" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D326" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D327" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D328" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D329" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D331" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D332" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D333" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D334" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D335" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D336" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D292" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D293" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D294" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D295" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D296" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D297" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D298" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D302" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D303" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D304" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D305" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D306" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D307" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D308" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D309" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D310" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D311" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D312" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D313" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D314" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D315" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D316" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D317" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D318" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D320" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D321" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D322" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D323" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D324" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D326" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D327" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D328" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D329" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D331" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D332" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D333" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D334" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D335" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D336" r:id="rId314"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21002,7 +20989,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15">
@@ -21012,7 +20999,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">

</xml_diff>